<commit_message>
[Modify][MOS_WORD_LEARN] Change mos word learn and excel learn file data
</commit_message>
<xml_diff>
--- a/Data/Excel_Learn/Excel_file_moi/12.xlsx
+++ b/Data/Excel_Learn/Excel_file_moi/12.xlsx
@@ -1,25 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7619693F-E432-4909-8929-DDFF4C78035D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30" yWindow="-30" windowWidth="20610" windowHeight="9195" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30" yWindow="-30" windowWidth="20610" windowHeight="9195" firstSheet="1" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Donor Contact Info" sheetId="5" r:id="rId1"/>
     <sheet name="Donor List" sheetId="1" r:id="rId2"/>
     <sheet name="Top Donors" sheetId="4" r:id="rId3"/>
     <sheet name="Demographics" sheetId="3" r:id="rId4"/>
-    <sheet name="Help (2)" sheetId="7" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="122211" fullCalcOnLoad="1" fullPrecision="1"/>
+  <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="244">
   <si>
     <t>First Name</t>
   </si>
@@ -751,25 +749,16 @@
   </si>
   <si>
     <t>Over 65</t>
-  </si>
-  <si>
-    <t>Help</t>
-  </si>
-  <si>
-    <t>1. Chọn worksheet "Donor List". Tô toàn bộ vùng từ A9 đến A11 -&gt; Chuột phải chọn Copy</t>
-  </si>
-  <si>
-    <t>2. Chuyển sang worksheet có tên "Top Donor". Chọn vào ô A2 sau đó nhấn chuột phải chọn Paste</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -792,14 +781,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -809,7 +790,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -817,44 +798,32 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" applyNumberFormat="0" fontId="3" applyFont="1" fillId="0" applyFill="0" borderId="1" applyBorder="1" applyProtection="0" applyAlignment="0"/>
-    <xf numFmtId="0" applyNumberFormat="0" fontId="1" applyFont="1" fillId="0" applyFill="0" borderId="0" applyBorder="0" applyProtection="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="8" applyNumberFormat="1" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" applyFont="1" fillId="0" borderId="0" xfId="2" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" applyFont="1" fillId="0" borderId="1" applyBorder="1" xfId="1"/>
-    <xf numFmtId="0" fontId="2" applyFont="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="3">
-    <cellStyle name="Heading 1" xfId="1" builtinId="16"/>
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Title" xfId="2" builtinId="15"/>
+    <cellStyle name="Title" xfId="1" builtinId="15"/>
   </cellStyles>
   <dxfs count="3">
     <dxf>
-      <numFmt numFmtId="12" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="12" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="12" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -944,63 +913,63 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:I47" totalsRowShown="0">
-  <autoFilter ref="A1:I47" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:I47" totalsRowShown="0">
+  <autoFilter ref="A1:I47"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="First Name"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Last Name"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Address"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="City"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="State"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Zip Code"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Work Phone"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Home Phone"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Email"/>
+    <tableColumn id="1" name="First Name"/>
+    <tableColumn id="2" name="Last Name"/>
+    <tableColumn id="3" name="Address"/>
+    <tableColumn id="4" name="City"/>
+    <tableColumn id="5" name="State"/>
+    <tableColumn id="6" name="Zip Code"/>
+    <tableColumn id="7" name="Work Phone"/>
+    <tableColumn id="8" name="Home Phone"/>
+    <tableColumn id="9" name="Email"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table2" displayName="Table2" ref="A7:C63" totalsRowShown="0">
-  <autoFilter ref="A7:C63" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A7:C63" totalsRowShown="0">
+  <autoFilter ref="A7:C63"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Name"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Annual Donations" dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Donation Level"/>
+    <tableColumn id="1" name="Name"/>
+    <tableColumn id="2" name="Annual Donations" dataDxfId="2"/>
+    <tableColumn id="3" name="Donation Level"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table4" displayName="Table4" ref="A1:D57" totalsRowShown="0">
-  <autoFilter ref="A1:D57" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Table4" displayName="Table4" ref="A1:D57" totalsRowShown="0">
+  <autoFilter ref="A1:D57"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Name"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Age Group"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Annual Donations" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Donation Level"/>
+    <tableColumn id="1" name="Name"/>
+    <tableColumn id="2" name="Age Group"/>
+    <tableColumn id="3" name="Annual Donations" dataDxfId="1"/>
+    <tableColumn id="4" name="Donation Level"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table5" displayName="Table5" ref="G3:H9" totalsRowShown="0">
-  <autoFilter ref="G3:H9" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Table5" displayName="Table5" ref="G3:H9" totalsRowShown="0">
+  <autoFilter ref="G3:H9"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Age Group"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Total Donations" dataDxfId="0"/>
+    <tableColumn id="1" name="Age Group"/>
+    <tableColumn id="2" name="Total Donations" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1038,9 +1007,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1075,7 +1044,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1110,7 +1079,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1283,1271 +1252,1270 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
-    <col min="2" max="2" bestFit="1" width="12.5703125" customWidth="1"/>
-    <col min="3" max="3" bestFit="1" width="18.5703125" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.85546875" customWidth="1"/>
     <col min="7" max="7" width="14.140625" customWidth="1"/>
     <col min="8" max="8" width="14.5703125" customWidth="1"/>
-    <col min="9" max="9" bestFit="1" width="28.28515625" customWidth="1"/>
+    <col min="9" max="9" width="28.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="0" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="0" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="0">
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2">
         <v>64044</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="I2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="0" t="s">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="0">
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3">
         <v>64044</v>
       </c>
-      <c r="H3" s="0" t="s">
+      <c r="H3" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="0" t="s">
+      <c r="I3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="0" t="s">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="0">
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4">
         <v>64030</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="G4" t="s">
         <v>24</v>
       </c>
-      <c r="H4" s="0" t="s">
+      <c r="H4" t="s">
         <v>25</v>
       </c>
-      <c r="I4" s="0" t="s">
+      <c r="I4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="0" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="0">
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5">
         <v>60063</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="G5" t="s">
         <v>31</v>
       </c>
-      <c r="I5" s="0" t="s">
+      <c r="I5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="0" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="0">
+      <c r="E6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6">
         <v>64030</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="G6" t="s">
         <v>24</v>
       </c>
-      <c r="H6" s="0" t="s">
+      <c r="H6" t="s">
         <v>25</v>
       </c>
-      <c r="I6" s="0" t="s">
+      <c r="I6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="0" t="s">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" t="s">
         <v>38</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="0">
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7">
         <v>64031</v>
       </c>
-      <c r="H7" s="0" t="s">
+      <c r="H7" t="s">
         <v>39</v>
       </c>
-      <c r="I7" s="0" t="s">
+      <c r="I7" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="0" t="s">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" s="0">
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8">
         <v>64045</v>
       </c>
-      <c r="H8" s="0" t="s">
+      <c r="H8" t="s">
         <v>44</v>
       </c>
-      <c r="I8" s="0" t="s">
+      <c r="I8" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="0" t="s">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" t="s">
         <v>47</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" s="0">
+      <c r="E9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9">
         <v>64044</v>
       </c>
-      <c r="G9" s="0" t="s">
+      <c r="G9" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="0" t="s">
+      <c r="I9" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="0" t="s">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>49</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" s="0">
+      <c r="E10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10">
         <v>64045</v>
       </c>
-      <c r="H10" s="0" t="s">
+      <c r="H10" t="s">
         <v>44</v>
       </c>
-      <c r="I10" s="0" t="s">
+      <c r="I10" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="0" t="s">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>52</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" t="s">
         <v>54</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" s="0">
+      <c r="E11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11">
         <v>64030</v>
       </c>
-      <c r="G11" s="0" t="s">
+      <c r="G11" t="s">
         <v>55</v>
       </c>
-      <c r="H11" s="0" t="s">
+      <c r="H11" t="s">
         <v>56</v>
       </c>
-      <c r="I11" s="0" t="s">
+      <c r="I11" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="0" t="s">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>58</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" t="s">
         <v>59</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" t="s">
         <v>38</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" s="0">
+      <c r="E12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12">
         <v>64031</v>
       </c>
-      <c r="H12" s="0" t="s">
+      <c r="H12" t="s">
         <v>39</v>
       </c>
-      <c r="I12" s="0" t="s">
+      <c r="I12" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="0" t="s">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>61</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" t="s">
         <v>62</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" t="s">
         <v>38</v>
       </c>
-      <c r="D13" s="0" t="s">
+      <c r="D13" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" s="0">
+      <c r="E13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13">
         <v>64031</v>
       </c>
-      <c r="H13" s="0" t="s">
+      <c r="H13" t="s">
         <v>39</v>
       </c>
-      <c r="I13" s="0" t="s">
+      <c r="I13" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="0" t="s">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>64</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" t="s">
         <v>62</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" t="s">
         <v>65</v>
       </c>
-      <c r="D14" s="0" t="s">
+      <c r="D14" t="s">
         <v>66</v>
       </c>
-      <c r="E14" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F14" s="0">
+      <c r="E14" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14">
         <v>64036</v>
       </c>
-      <c r="H14" s="0" t="s">
+      <c r="H14" t="s">
         <v>67</v>
       </c>
-      <c r="I14" s="0" t="s">
+      <c r="I14" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="0" t="s">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>69</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" t="s">
         <v>70</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" t="s">
         <v>43</v>
       </c>
-      <c r="D15" s="0" t="s">
+      <c r="D15" t="s">
         <v>12</v>
       </c>
-      <c r="E15" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" s="0">
+      <c r="E15" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15">
         <v>64045</v>
       </c>
-      <c r="H15" s="0" t="s">
+      <c r="H15" t="s">
         <v>44</v>
       </c>
-      <c r="I15" s="0" t="s">
+      <c r="I15" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="0" t="s">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>72</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" t="s">
         <v>73</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" t="s">
         <v>54</v>
       </c>
-      <c r="D16" s="0" t="s">
+      <c r="D16" t="s">
         <v>12</v>
       </c>
-      <c r="E16" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F16" s="0">
+      <c r="E16" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16">
         <v>64030</v>
       </c>
-      <c r="G16" s="0" t="s">
+      <c r="G16" t="s">
         <v>55</v>
       </c>
-      <c r="H16" s="0" t="s">
+      <c r="H16" t="s">
         <v>56</v>
       </c>
-      <c r="I16" s="0" t="s">
+      <c r="I16" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="0" t="s">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>75</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" t="s">
         <v>76</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" t="s">
         <v>29</v>
       </c>
-      <c r="D17" s="0" t="s">
+      <c r="D17" t="s">
         <v>30</v>
       </c>
-      <c r="E17" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F17" s="0">
+      <c r="E17" t="s">
+        <v>13</v>
+      </c>
+      <c r="F17">
         <v>60063</v>
       </c>
-      <c r="G17" s="0" t="s">
+      <c r="G17" t="s">
         <v>31</v>
       </c>
-      <c r="I17" s="0" t="s">
+      <c r="I17" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="0" t="s">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>78</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" t="s">
         <v>79</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="C18" t="s">
         <v>80</v>
       </c>
-      <c r="D18" s="0" t="s">
+      <c r="D18" t="s">
         <v>12</v>
       </c>
-      <c r="E18" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F18" s="0">
+      <c r="E18" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18">
         <v>64044</v>
       </c>
-      <c r="H18" s="0" t="s">
+      <c r="H18" t="s">
         <v>81</v>
       </c>
-      <c r="I18" s="0" t="s">
+      <c r="I18" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="0" t="s">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>83</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" t="s">
         <v>84</v>
       </c>
-      <c r="C19" s="0" t="s">
+      <c r="C19" t="s">
         <v>85</v>
       </c>
-      <c r="D19" s="0" t="s">
+      <c r="D19" t="s">
         <v>66</v>
       </c>
-      <c r="E19" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F19" s="0">
+      <c r="E19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19">
         <v>64036</v>
       </c>
-      <c r="H19" s="0" t="s">
+      <c r="H19" t="s">
         <v>86</v>
       </c>
-      <c r="I19" s="0" t="s">
+      <c r="I19" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="0" t="s">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>88</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" t="s">
         <v>89</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="C20" t="s">
         <v>65</v>
       </c>
-      <c r="D20" s="0" t="s">
+      <c r="D20" t="s">
         <v>66</v>
       </c>
-      <c r="E20" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F20" s="0">
+      <c r="E20" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20">
         <v>64036</v>
       </c>
-      <c r="H20" s="0" t="s">
+      <c r="H20" t="s">
         <v>67</v>
       </c>
-      <c r="I20" s="0" t="s">
+      <c r="I20" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="0" t="s">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>91</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" t="s">
         <v>92</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="C21" t="s">
         <v>18</v>
       </c>
-      <c r="D21" s="0" t="s">
+      <c r="D21" t="s">
         <v>12</v>
       </c>
-      <c r="E21" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F21" s="0">
+      <c r="E21" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21">
         <v>64044</v>
       </c>
-      <c r="H21" s="0" t="s">
+      <c r="H21" t="s">
         <v>19</v>
       </c>
-      <c r="I21" s="0" t="s">
+      <c r="I21" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="0" t="s">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>94</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="B22" t="s">
         <v>95</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="C22" t="s">
         <v>11</v>
       </c>
-      <c r="D22" s="0" t="s">
+      <c r="D22" t="s">
         <v>12</v>
       </c>
-      <c r="E22" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F22" s="0">
+      <c r="E22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F22">
         <v>64044</v>
       </c>
-      <c r="G22" s="0" t="s">
+      <c r="G22" t="s">
         <v>14</v>
       </c>
-      <c r="I22" s="0" t="s">
+      <c r="I22" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="0" t="s">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>97</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" t="s">
         <v>98</v>
       </c>
-      <c r="C23" s="0" t="s">
+      <c r="C23" t="s">
         <v>85</v>
       </c>
-      <c r="D23" s="0" t="s">
+      <c r="D23" t="s">
         <v>66</v>
       </c>
-      <c r="E23" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F23" s="0">
+      <c r="E23" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23">
         <v>64036</v>
       </c>
-      <c r="H23" s="0" t="s">
+      <c r="H23" t="s">
         <v>86</v>
       </c>
-      <c r="I23" s="0" t="s">
+      <c r="I23" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="0" t="s">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>100</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" t="s">
         <v>101</v>
       </c>
-      <c r="C24" s="0" t="s">
+      <c r="C24" t="s">
         <v>54</v>
       </c>
-      <c r="D24" s="0" t="s">
+      <c r="D24" t="s">
         <v>12</v>
       </c>
-      <c r="E24" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F24" s="0">
+      <c r="E24" t="s">
+        <v>13</v>
+      </c>
+      <c r="F24">
         <v>64030</v>
       </c>
-      <c r="G24" s="0" t="s">
+      <c r="G24" t="s">
         <v>55</v>
       </c>
-      <c r="H24" s="0" t="s">
+      <c r="H24" t="s">
         <v>56</v>
       </c>
-      <c r="I24" s="0" t="s">
+      <c r="I24" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="0" t="s">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>103</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" t="s">
         <v>104</v>
       </c>
-      <c r="C25" s="0" t="s">
+      <c r="C25" t="s">
         <v>11</v>
       </c>
-      <c r="D25" s="0" t="s">
+      <c r="D25" t="s">
         <v>12</v>
       </c>
-      <c r="E25" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F25" s="0">
+      <c r="E25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F25">
         <v>64044</v>
       </c>
-      <c r="G25" s="0" t="s">
+      <c r="G25" t="s">
         <v>14</v>
       </c>
-      <c r="I25" s="0" t="s">
+      <c r="I25" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="0" t="s">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>106</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="B26" t="s">
         <v>107</v>
       </c>
-      <c r="C26" s="0" t="s">
+      <c r="C26" t="s">
         <v>85</v>
       </c>
-      <c r="D26" s="0" t="s">
+      <c r="D26" t="s">
         <v>66</v>
       </c>
-      <c r="E26" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F26" s="0">
+      <c r="E26" t="s">
+        <v>13</v>
+      </c>
+      <c r="F26">
         <v>64036</v>
       </c>
-      <c r="H26" s="0" t="s">
+      <c r="H26" t="s">
         <v>86</v>
       </c>
-      <c r="I26" s="0" t="s">
+      <c r="I26" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="0" t="s">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>109</v>
       </c>
-      <c r="B27" s="0" t="s">
+      <c r="B27" t="s">
         <v>110</v>
       </c>
-      <c r="C27" s="0" t="s">
+      <c r="C27" t="s">
         <v>80</v>
       </c>
-      <c r="D27" s="0" t="s">
+      <c r="D27" t="s">
         <v>12</v>
       </c>
-      <c r="E27" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F27" s="0">
+      <c r="E27" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27">
         <v>64044</v>
       </c>
-      <c r="H27" s="0" t="s">
+      <c r="H27" t="s">
         <v>81</v>
       </c>
-      <c r="I27" s="0" t="s">
+      <c r="I27" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="0" t="s">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>112</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="B28" t="s">
         <v>113</v>
       </c>
-      <c r="C28" s="0" t="s">
+      <c r="C28" t="s">
         <v>54</v>
       </c>
-      <c r="D28" s="0" t="s">
+      <c r="D28" t="s">
         <v>12</v>
       </c>
-      <c r="E28" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F28" s="0">
+      <c r="E28" t="s">
+        <v>13</v>
+      </c>
+      <c r="F28">
         <v>64030</v>
       </c>
-      <c r="G28" s="0" t="s">
+      <c r="G28" t="s">
         <v>55</v>
       </c>
-      <c r="H28" s="0" t="s">
+      <c r="H28" t="s">
         <v>56</v>
       </c>
-      <c r="I28" s="0" t="s">
+      <c r="I28" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="0" t="s">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>115</v>
       </c>
-      <c r="B29" s="0" t="s">
+      <c r="B29" t="s">
         <v>116</v>
       </c>
-      <c r="C29" s="0" t="s">
+      <c r="C29" t="s">
         <v>65</v>
       </c>
-      <c r="D29" s="0" t="s">
+      <c r="D29" t="s">
         <v>66</v>
       </c>
-      <c r="E29" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F29" s="0">
+      <c r="E29" t="s">
+        <v>13</v>
+      </c>
+      <c r="F29">
         <v>64036</v>
       </c>
-      <c r="H29" s="0" t="s">
+      <c r="H29" t="s">
         <v>67</v>
       </c>
-      <c r="I29" s="0" t="s">
+      <c r="I29" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="0" t="s">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>118</v>
       </c>
-      <c r="B30" s="0" t="s">
+      <c r="B30" t="s">
         <v>119</v>
       </c>
-      <c r="C30" s="0" t="s">
+      <c r="C30" t="s">
         <v>85</v>
       </c>
-      <c r="D30" s="0" t="s">
+      <c r="D30" t="s">
         <v>66</v>
       </c>
-      <c r="E30" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F30" s="0">
+      <c r="E30" t="s">
+        <v>13</v>
+      </c>
+      <c r="F30">
         <v>64036</v>
       </c>
-      <c r="H30" s="0" t="s">
+      <c r="H30" t="s">
         <v>86</v>
       </c>
-      <c r="I30" s="0" t="s">
+      <c r="I30" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="0" t="s">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>121</v>
       </c>
-      <c r="B31" s="0" t="s">
+      <c r="B31" t="s">
         <v>122</v>
       </c>
-      <c r="C31" s="0" t="s">
+      <c r="C31" t="s">
         <v>65</v>
       </c>
-      <c r="D31" s="0" t="s">
+      <c r="D31" t="s">
         <v>66</v>
       </c>
-      <c r="E31" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F31" s="0">
+      <c r="E31" t="s">
+        <v>13</v>
+      </c>
+      <c r="F31">
         <v>64036</v>
       </c>
-      <c r="H31" s="0" t="s">
+      <c r="H31" t="s">
         <v>67</v>
       </c>
-      <c r="I31" s="0" t="s">
+      <c r="I31" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="0" t="s">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>124</v>
       </c>
-      <c r="B32" s="0" t="s">
+      <c r="B32" t="s">
         <v>125</v>
       </c>
-      <c r="C32" s="0" t="s">
+      <c r="C32" t="s">
         <v>23</v>
       </c>
-      <c r="D32" s="0" t="s">
+      <c r="D32" t="s">
         <v>12</v>
       </c>
-      <c r="E32" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F32" s="0">
+      <c r="E32" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32">
         <v>64030</v>
       </c>
-      <c r="G32" s="0" t="s">
+      <c r="G32" t="s">
         <v>24</v>
       </c>
-      <c r="H32" s="0" t="s">
+      <c r="H32" t="s">
         <v>25</v>
       </c>
-      <c r="I32" s="0" t="s">
+      <c r="I32" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="0" t="s">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>127</v>
       </c>
-      <c r="B33" s="0" t="s">
+      <c r="B33" t="s">
         <v>128</v>
       </c>
-      <c r="C33" s="0" t="s">
+      <c r="C33" t="s">
         <v>43</v>
       </c>
-      <c r="D33" s="0" t="s">
+      <c r="D33" t="s">
         <v>12</v>
       </c>
-      <c r="E33" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F33" s="0">
+      <c r="E33" t="s">
+        <v>13</v>
+      </c>
+      <c r="F33">
         <v>64045</v>
       </c>
-      <c r="H33" s="0" t="s">
+      <c r="H33" t="s">
         <v>44</v>
       </c>
-      <c r="I33" s="0" t="s">
+      <c r="I33" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="0" t="s">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>130</v>
       </c>
-      <c r="B34" s="0" t="s">
+      <c r="B34" t="s">
         <v>131</v>
       </c>
-      <c r="C34" s="0" t="s">
+      <c r="C34" t="s">
         <v>85</v>
       </c>
-      <c r="D34" s="0" t="s">
+      <c r="D34" t="s">
         <v>66</v>
       </c>
-      <c r="E34" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F34" s="0">
+      <c r="E34" t="s">
+        <v>13</v>
+      </c>
+      <c r="F34">
         <v>64036</v>
       </c>
-      <c r="H34" s="0" t="s">
+      <c r="H34" t="s">
         <v>86</v>
       </c>
-      <c r="I34" s="0" t="s">
+      <c r="I34" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="0" t="s">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>61</v>
       </c>
-      <c r="B35" s="0" t="s">
+      <c r="B35" t="s">
         <v>133</v>
       </c>
-      <c r="C35" s="0" t="s">
+      <c r="C35" t="s">
         <v>23</v>
       </c>
-      <c r="D35" s="0" t="s">
+      <c r="D35" t="s">
         <v>12</v>
       </c>
-      <c r="E35" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F35" s="0">
+      <c r="E35" t="s">
+        <v>13</v>
+      </c>
+      <c r="F35">
         <v>64030</v>
       </c>
-      <c r="G35" s="0" t="s">
+      <c r="G35" t="s">
         <v>24</v>
       </c>
-      <c r="H35" s="0" t="s">
+      <c r="H35" t="s">
         <v>25</v>
       </c>
-      <c r="I35" s="0" t="s">
+      <c r="I35" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="0" t="s">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>135</v>
       </c>
-      <c r="B36" s="0" t="s">
+      <c r="B36" t="s">
         <v>136</v>
       </c>
-      <c r="C36" s="0" t="s">
+      <c r="C36" t="s">
         <v>18</v>
       </c>
-      <c r="D36" s="0" t="s">
+      <c r="D36" t="s">
         <v>12</v>
       </c>
-      <c r="E36" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F36" s="0">
+      <c r="E36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F36">
         <v>64044</v>
       </c>
-      <c r="H36" s="0" t="s">
+      <c r="H36" t="s">
         <v>19</v>
       </c>
-      <c r="I36" s="0" t="s">
+      <c r="I36" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="0" t="s">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>138</v>
       </c>
-      <c r="B37" s="0" t="s">
+      <c r="B37" t="s">
         <v>139</v>
       </c>
-      <c r="C37" s="0" t="s">
+      <c r="C37" t="s">
         <v>29</v>
       </c>
-      <c r="D37" s="0" t="s">
+      <c r="D37" t="s">
         <v>30</v>
       </c>
-      <c r="E37" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F37" s="0">
+      <c r="E37" t="s">
+        <v>13</v>
+      </c>
+      <c r="F37">
         <v>60063</v>
       </c>
-      <c r="G37" s="0" t="s">
+      <c r="G37" t="s">
         <v>31</v>
       </c>
-      <c r="I37" s="0" t="s">
+      <c r="I37" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="0" t="s">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>141</v>
       </c>
-      <c r="B38" s="0" t="s">
+      <c r="B38" t="s">
         <v>142</v>
       </c>
-      <c r="C38" s="0" t="s">
+      <c r="C38" t="s">
         <v>65</v>
       </c>
-      <c r="D38" s="0" t="s">
+      <c r="D38" t="s">
         <v>66</v>
       </c>
-      <c r="E38" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F38" s="0">
+      <c r="E38" t="s">
+        <v>13</v>
+      </c>
+      <c r="F38">
         <v>64036</v>
       </c>
-      <c r="H38" s="0" t="s">
+      <c r="H38" t="s">
         <v>67</v>
       </c>
-      <c r="I38" s="0" t="s">
+      <c r="I38" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="0" t="s">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>144</v>
       </c>
-      <c r="B39" s="0" t="s">
+      <c r="B39" t="s">
         <v>145</v>
       </c>
-      <c r="C39" s="0" t="s">
+      <c r="C39" t="s">
         <v>11</v>
       </c>
-      <c r="D39" s="0" t="s">
+      <c r="D39" t="s">
         <v>12</v>
       </c>
-      <c r="E39" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F39" s="0">
+      <c r="E39" t="s">
+        <v>13</v>
+      </c>
+      <c r="F39">
         <v>64044</v>
       </c>
-      <c r="G39" s="0" t="s">
+      <c r="G39" t="s">
         <v>14</v>
       </c>
-      <c r="I39" s="0" t="s">
+      <c r="I39" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="0" t="s">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>33</v>
       </c>
-      <c r="B40" s="0" t="s">
+      <c r="B40" t="s">
         <v>145</v>
       </c>
-      <c r="C40" s="0" t="s">
+      <c r="C40" t="s">
         <v>80</v>
       </c>
-      <c r="D40" s="0" t="s">
+      <c r="D40" t="s">
         <v>12</v>
       </c>
-      <c r="E40" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F40" s="0">
+      <c r="E40" t="s">
+        <v>13</v>
+      </c>
+      <c r="F40">
         <v>64044</v>
       </c>
-      <c r="H40" s="0" t="s">
+      <c r="H40" t="s">
         <v>81</v>
       </c>
-      <c r="I40" s="0" t="s">
+      <c r="I40" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="0" t="s">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>147</v>
       </c>
-      <c r="B41" s="0" t="s">
+      <c r="B41" t="s">
         <v>148</v>
       </c>
-      <c r="C41" s="0" t="s">
+      <c r="C41" t="s">
         <v>85</v>
       </c>
-      <c r="D41" s="0" t="s">
+      <c r="D41" t="s">
         <v>66</v>
       </c>
-      <c r="E41" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F41" s="0">
+      <c r="E41" t="s">
+        <v>13</v>
+      </c>
+      <c r="F41">
         <v>64036</v>
       </c>
-      <c r="H41" s="0" t="s">
+      <c r="H41" t="s">
         <v>86</v>
       </c>
-      <c r="I41" s="0" t="s">
+      <c r="I41" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="0" t="s">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>150</v>
       </c>
-      <c r="B42" s="0" t="s">
+      <c r="B42" t="s">
         <v>151</v>
       </c>
-      <c r="C42" s="0" t="s">
+      <c r="C42" t="s">
         <v>38</v>
       </c>
-      <c r="D42" s="0" t="s">
+      <c r="D42" t="s">
         <v>12</v>
       </c>
-      <c r="E42" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F42" s="0">
+      <c r="E42" t="s">
+        <v>13</v>
+      </c>
+      <c r="F42">
         <v>64031</v>
       </c>
-      <c r="H42" s="0" t="s">
+      <c r="H42" t="s">
         <v>39</v>
       </c>
-      <c r="I42" s="0" t="s">
+      <c r="I42" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="0" t="s">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>153</v>
       </c>
-      <c r="B43" s="0" t="s">
+      <c r="B43" t="s">
         <v>154</v>
       </c>
-      <c r="C43" s="0" t="s">
+      <c r="C43" t="s">
         <v>38</v>
       </c>
-      <c r="D43" s="0" t="s">
+      <c r="D43" t="s">
         <v>12</v>
       </c>
-      <c r="E43" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F43" s="0">
+      <c r="E43" t="s">
+        <v>13</v>
+      </c>
+      <c r="F43">
         <v>64031</v>
       </c>
-      <c r="H43" s="0" t="s">
+      <c r="H43" t="s">
         <v>39</v>
       </c>
-      <c r="I43" s="0" t="s">
+      <c r="I43" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="0" t="s">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>145</v>
       </c>
-      <c r="B44" s="0" t="s">
+      <c r="B44" t="s">
         <v>156</v>
       </c>
-      <c r="C44" s="0" t="s">
+      <c r="C44" t="s">
         <v>29</v>
       </c>
-      <c r="D44" s="0" t="s">
+      <c r="D44" t="s">
         <v>30</v>
       </c>
-      <c r="E44" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F44" s="0">
+      <c r="E44" t="s">
+        <v>13</v>
+      </c>
+      <c r="F44">
         <v>60063</v>
       </c>
-      <c r="G44" s="0" t="s">
+      <c r="G44" t="s">
         <v>31</v>
       </c>
-      <c r="I44" s="0" t="s">
+      <c r="I44" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="0" t="s">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>158</v>
       </c>
-      <c r="B45" s="0" t="s">
+      <c r="B45" t="s">
         <v>159</v>
       </c>
-      <c r="C45" s="0" t="s">
+      <c r="C45" t="s">
         <v>65</v>
       </c>
-      <c r="D45" s="0" t="s">
+      <c r="D45" t="s">
         <v>66</v>
       </c>
-      <c r="E45" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F45" s="0">
+      <c r="E45" t="s">
+        <v>13</v>
+      </c>
+      <c r="F45">
         <v>64036</v>
       </c>
-      <c r="H45" s="0" t="s">
+      <c r="H45" t="s">
         <v>67</v>
       </c>
-      <c r="I45" s="0" t="s">
+      <c r="I45" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="0" t="s">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>161</v>
       </c>
-      <c r="B46" s="0" t="s">
+      <c r="B46" t="s">
         <v>162</v>
       </c>
-      <c r="C46" s="0" t="s">
+      <c r="C46" t="s">
         <v>80</v>
       </c>
-      <c r="D46" s="0" t="s">
+      <c r="D46" t="s">
         <v>12</v>
       </c>
-      <c r="E46" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F46" s="0">
+      <c r="E46" t="s">
+        <v>13</v>
+      </c>
+      <c r="F46">
         <v>64044</v>
       </c>
-      <c r="H46" s="0" t="s">
+      <c r="H46" t="s">
         <v>81</v>
       </c>
-      <c r="I46" s="0" t="s">
+      <c r="I46" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="0" t="s">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>164</v>
       </c>
-      <c r="B47" s="0" t="s">
+      <c r="B47" t="s">
         <v>165</v>
       </c>
-      <c r="C47" s="0" t="s">
+      <c r="C47" t="s">
         <v>29</v>
       </c>
-      <c r="D47" s="0" t="s">
+      <c r="D47" t="s">
         <v>30</v>
       </c>
-      <c r="E47" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F47" s="0">
+      <c r="E47" t="s">
+        <v>13</v>
+      </c>
+      <c r="F47">
         <v>60063</v>
       </c>
-      <c r="G47" s="0" t="s">
+      <c r="G47" t="s">
         <v>31</v>
       </c>
-      <c r="I47" s="0" t="s">
+      <c r="I47" t="s">
         <v>166</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -2555,715 +2523,713 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A6:H63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" bestFit="1" width="22" customWidth="1"/>
+    <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.85546875" customWidth="1"/>
     <col min="3" max="3" width="16.42578125" customWidth="1"/>
-    <col min="8" max="8" bestFit="1" width="18.42578125" customWidth="1"/>
+    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="6" ht="19.5">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:8" ht="19.5" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="0" t="s">
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>168</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" t="s">
         <v>169</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" t="s">
         <v>170</v>
       </c>
-      <c r="G7" s="0" t="s">
+      <c r="G7" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="0" t="s">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>172</v>
       </c>
       <c r="B8" s="1">
         <v>84</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" t="s">
         <v>173</v>
       </c>
-      <c r="G8" s="0" t="s">
+      <c r="G8" t="s">
         <v>174</v>
       </c>
-      <c r="H8" s="0" t="s">
+      <c r="H8" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="0" t="s">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>176</v>
       </c>
       <c r="B9" s="1">
         <v>88</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" t="s">
         <v>173</v>
       </c>
-      <c r="G9" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="H9" s="0">
+      <c r="G9" t="s">
+        <v>177</v>
+      </c>
+      <c r="H9">
         <v>1000</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="0" t="s">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>178</v>
       </c>
       <c r="B10" s="1">
         <v>91</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" t="s">
         <v>173</v>
       </c>
-      <c r="G10" s="0" t="s">
+      <c r="G10" t="s">
         <v>179</v>
       </c>
-      <c r="H10" s="0">
+      <c r="H10">
         <v>500</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="0" t="s">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>180</v>
       </c>
       <c r="B11" s="1">
         <v>125</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" t="s">
         <v>173</v>
       </c>
-      <c r="G11" s="0" t="s">
+      <c r="G11" t="s">
         <v>181</v>
       </c>
-      <c r="H11" s="0">
+      <c r="H11">
         <v>250</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="0" t="s">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>182</v>
       </c>
       <c r="B12" s="1">
         <v>142</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" t="s">
         <v>173</v>
       </c>
-      <c r="G12" s="0" t="s">
+      <c r="G12" t="s">
         <v>173</v>
       </c>
-      <c r="H12" s="0">
+      <c r="H12">
         <v>10</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="0" t="s">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>183</v>
       </c>
       <c r="B13" s="1">
         <v>166</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="0" t="s">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>184</v>
       </c>
       <c r="B14" s="1">
         <v>226</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="0" t="s">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>185</v>
       </c>
       <c r="B15" s="1">
         <v>238</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="0" t="s">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>186</v>
       </c>
       <c r="B16" s="1">
         <v>259</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="0" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>187</v>
       </c>
       <c r="B17" s="1">
         <v>301</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="0" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>188</v>
       </c>
       <c r="B18" s="1">
         <v>301</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="C18" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="0" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>189</v>
       </c>
       <c r="B19" s="1">
         <v>322</v>
       </c>
-      <c r="C19" s="0" t="s">
+      <c r="C19" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="0" t="s">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>190</v>
       </c>
       <c r="B20" s="1">
         <v>330</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="C20" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="0" t="s">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>191</v>
       </c>
       <c r="B21" s="1">
         <v>334</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="C21" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="0" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>192</v>
       </c>
       <c r="B22" s="1">
         <v>393</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="C22" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="0" t="s">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>193</v>
       </c>
       <c r="B23" s="1">
         <v>433</v>
       </c>
-      <c r="C23" s="0" t="s">
+      <c r="C23" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="0" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>194</v>
       </c>
       <c r="B24" s="1">
         <v>453</v>
       </c>
-      <c r="C24" s="0" t="s">
+      <c r="C24" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="0" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>195</v>
       </c>
       <c r="B25" s="1">
         <v>467</v>
       </c>
-      <c r="C25" s="0" t="s">
+      <c r="C25" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="0" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>196</v>
       </c>
       <c r="B26" s="1">
         <v>557</v>
       </c>
-      <c r="C26" s="0" t="s">
+      <c r="C26" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="0" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>197</v>
       </c>
       <c r="B27" s="1">
         <v>564</v>
       </c>
-      <c r="C27" s="0" t="s">
+      <c r="C27" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="0" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>198</v>
       </c>
       <c r="B28" s="1">
         <v>577</v>
       </c>
-      <c r="C28" s="0" t="s">
+      <c r="C28" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="0" t="s">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>199</v>
       </c>
       <c r="B29" s="1">
         <v>580</v>
       </c>
-      <c r="C29" s="0" t="s">
+      <c r="C29" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="0" t="s">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>200</v>
       </c>
       <c r="B30" s="1">
         <v>581</v>
       </c>
-      <c r="C30" s="0" t="s">
+      <c r="C30" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="0" t="s">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>201</v>
       </c>
       <c r="B31" s="1">
         <v>656</v>
       </c>
-      <c r="C31" s="0" t="s">
+      <c r="C31" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="0" t="s">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>202</v>
       </c>
       <c r="B32" s="1">
         <v>706</v>
       </c>
-      <c r="C32" s="0" t="s">
+      <c r="C32" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="0" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>203</v>
       </c>
       <c r="B33" s="1">
         <v>722</v>
       </c>
-      <c r="C33" s="0" t="s">
+      <c r="C33" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="0" t="s">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>204</v>
       </c>
       <c r="B34" s="1">
         <v>782</v>
       </c>
-      <c r="C34" s="0" t="s">
+      <c r="C34" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="0" t="s">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>205</v>
       </c>
       <c r="B35" s="1">
         <v>910</v>
       </c>
-      <c r="C35" s="0" t="s">
+      <c r="C35" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="0" t="s">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>206</v>
       </c>
       <c r="B36" s="1">
         <v>951</v>
       </c>
-      <c r="C36" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="0" t="s">
+      <c r="C36" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>207</v>
       </c>
       <c r="B37" s="1">
         <v>1000</v>
       </c>
-      <c r="C37" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="0" t="s">
+      <c r="C37" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>208</v>
       </c>
       <c r="B38" s="1">
         <v>1001</v>
       </c>
-      <c r="C38" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="0" t="s">
+      <c r="C38" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>209</v>
       </c>
       <c r="B39" s="1">
         <v>1018</v>
       </c>
-      <c r="C39" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="0" t="s">
+      <c r="C39" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>210</v>
       </c>
       <c r="B40" s="1">
         <v>1022</v>
       </c>
-      <c r="C40" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="0" t="s">
+      <c r="C40" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>211</v>
       </c>
       <c r="B41" s="1">
         <v>1059</v>
       </c>
-      <c r="C41" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="0" t="s">
+      <c r="C41" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>212</v>
       </c>
       <c r="B42" s="1">
         <v>1191</v>
       </c>
-      <c r="C42" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="0" t="s">
+      <c r="C42" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>213</v>
       </c>
       <c r="B43" s="1">
         <v>1208</v>
       </c>
-      <c r="C43" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="0" t="s">
+      <c r="C43" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>214</v>
       </c>
       <c r="B44" s="1">
         <v>1215</v>
       </c>
-      <c r="C44" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="0" t="s">
+      <c r="C44" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>215</v>
       </c>
       <c r="B45" s="1">
         <v>1218</v>
       </c>
-      <c r="C45" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="0" t="s">
+      <c r="C45" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>216</v>
       </c>
       <c r="B46" s="1">
         <v>1218</v>
       </c>
-      <c r="C46" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="0" t="s">
+      <c r="C46" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>217</v>
       </c>
       <c r="B47" s="1">
         <v>1236</v>
       </c>
-      <c r="C47" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="0" t="s">
+      <c r="C47" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>218</v>
       </c>
       <c r="B48" s="1">
         <v>1236</v>
       </c>
-      <c r="C48" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="0" t="s">
+      <c r="C48" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
         <v>219</v>
       </c>
       <c r="B49" s="1">
         <v>1247</v>
       </c>
-      <c r="C49" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="0" t="s">
+      <c r="C49" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
         <v>220</v>
       </c>
       <c r="B50" s="1">
         <v>1256</v>
       </c>
-      <c r="C50" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="0" t="s">
+      <c r="C50" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
         <v>221</v>
       </c>
       <c r="B51" s="1">
         <v>1351</v>
       </c>
-      <c r="C51" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="0" t="s">
+      <c r="C51" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
         <v>222</v>
       </c>
       <c r="B52" s="1">
         <v>1356</v>
       </c>
-      <c r="C52" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="0" t="s">
+      <c r="C52" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
         <v>223</v>
       </c>
       <c r="B53" s="1">
         <v>1399</v>
       </c>
-      <c r="C53" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="0" t="s">
+      <c r="C53" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
         <v>224</v>
       </c>
       <c r="B54" s="1">
         <v>1425</v>
       </c>
-      <c r="C54" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="0" t="s">
+      <c r="C54" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
         <v>225</v>
       </c>
       <c r="B55" s="1">
         <v>1456</v>
       </c>
-      <c r="C55" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="0" t="s">
+      <c r="C55" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
         <v>226</v>
       </c>
       <c r="B56" s="1">
         <v>1527</v>
       </c>
-      <c r="C56" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="0" t="s">
+      <c r="C56" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
         <v>227</v>
       </c>
       <c r="B57" s="1">
         <v>1581</v>
       </c>
-      <c r="C57" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="0" t="s">
+      <c r="C57" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
         <v>228</v>
       </c>
       <c r="B58" s="1">
         <v>1656</v>
       </c>
-      <c r="C58" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="0" t="s">
+      <c r="C58" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
         <v>229</v>
       </c>
       <c r="B59" s="1">
         <v>1802</v>
       </c>
-      <c r="C59" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="0" t="s">
+      <c r="C59" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
         <v>230</v>
       </c>
       <c r="B60" s="1">
         <v>1816</v>
       </c>
-      <c r="C60" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="0" t="s">
+      <c r="C60" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
         <v>231</v>
       </c>
       <c r="B61" s="1">
         <v>1829</v>
       </c>
-      <c r="C61" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="0" t="s">
+      <c r="C61" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
         <v>232</v>
       </c>
       <c r="B62" s="1">
         <v>1841</v>
       </c>
-      <c r="C62" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="0" t="s">
+      <c r="C62" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
         <v>233</v>
       </c>
       <c r="B63" s="1">
         <v>1906</v>
       </c>
-      <c r="C63" s="0" t="s">
+      <c r="C63" t="s">
         <v>177</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells>
+  <mergeCells count="1">
     <mergeCell ref="A6:C6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
-  <headerFooter/>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" ht="22.5">
+    <row r="1" spans="1:1" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>234</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3274,886 +3240,854 @@
     <col min="8" max="8" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="0" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>168</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" t="s">
         <v>235</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" t="s">
         <v>169</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="0" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>176</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" t="s">
         <v>236</v>
       </c>
       <c r="C2" s="1">
         <v>88</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" t="s">
         <v>173</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="0" t="s">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>185</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" t="s">
         <v>236</v>
       </c>
       <c r="C3" s="1">
         <v>238</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" t="s">
         <v>173</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="G3" t="s">
         <v>235</v>
       </c>
-      <c r="H3" s="0" t="s">
+      <c r="H3" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="0" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>191</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" t="s">
         <v>236</v>
       </c>
       <c r="C4" s="1">
         <v>334</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" t="s">
         <v>181</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="G4" t="s">
         <v>239</v>
       </c>
       <c r="H4" s="1">
         <v>10151</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="0" t="s">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>197</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" t="s">
         <v>236</v>
       </c>
       <c r="C5" s="1">
         <v>564</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" t="s">
         <v>179</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="G5" t="s">
         <v>236</v>
       </c>
       <c r="H5" s="1">
         <v>5708</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="0" t="s">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>221</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" t="s">
         <v>236</v>
       </c>
       <c r="C6" s="1">
         <v>1351</v>
       </c>
-      <c r="D6" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="G6" s="0" t="s">
+      <c r="D6" t="s">
+        <v>177</v>
+      </c>
+      <c r="G6" t="s">
         <v>240</v>
       </c>
       <c r="H6" s="1">
         <v>4278</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="0" t="s">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>227</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" t="s">
         <v>236</v>
       </c>
       <c r="C7" s="1">
         <v>1581</v>
       </c>
-      <c r="D7" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="G7" s="0" t="s">
+      <c r="D7" t="s">
+        <v>177</v>
+      </c>
+      <c r="G7" t="s">
         <v>241</v>
       </c>
       <c r="H7" s="1">
         <v>6661</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="0" t="s">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>211</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" t="s">
         <v>236</v>
       </c>
       <c r="C8" s="1">
         <v>1059</v>
       </c>
-      <c r="D8" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="G8" s="0" t="s">
+      <c r="D8" t="s">
+        <v>177</v>
+      </c>
+      <c r="G8" t="s">
         <v>242</v>
       </c>
       <c r="H8" s="1">
         <v>9373</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="0" t="s">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>200</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" t="s">
         <v>236</v>
       </c>
       <c r="C9" s="1">
         <v>581</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" t="s">
         <v>179</v>
       </c>
-      <c r="G9" s="0" t="s">
+      <c r="G9" t="s">
         <v>243</v>
       </c>
       <c r="H9" s="1">
         <v>13150</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="0" t="s">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>178</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" t="s">
         <v>240</v>
       </c>
       <c r="C10" s="1">
         <v>91</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="0" t="s">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>192</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" t="s">
         <v>240</v>
       </c>
       <c r="C11" s="1">
         <v>393</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="0" t="s">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>204</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" t="s">
         <v>240</v>
       </c>
       <c r="C12" s="1">
         <v>782</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="0" t="s">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>222</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" t="s">
         <v>240</v>
       </c>
       <c r="C13" s="1">
         <v>1356</v>
       </c>
-      <c r="D13" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="0" t="s">
+      <c r="D13" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>228</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" t="s">
         <v>240</v>
       </c>
       <c r="C14" s="1">
         <v>1656</v>
       </c>
-      <c r="D14" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="0" t="s">
+      <c r="D14" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>187</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" t="s">
         <v>241</v>
       </c>
       <c r="C15" s="1">
         <v>301</v>
       </c>
-      <c r="D15" s="0" t="s">
+      <c r="D15" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="0" t="s">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>193</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" t="s">
         <v>241</v>
       </c>
       <c r="C16" s="1">
         <v>433</v>
       </c>
-      <c r="D16" s="0" t="s">
+      <c r="D16" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="0" t="s">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>199</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" t="s">
         <v>241</v>
       </c>
       <c r="C17" s="1">
         <v>580</v>
       </c>
-      <c r="D17" s="0" t="s">
+      <c r="D17" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="0" t="s">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>205</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" t="s">
         <v>241</v>
       </c>
       <c r="C18" s="1">
         <v>910</v>
       </c>
-      <c r="D18" s="0" t="s">
+      <c r="D18" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="0" t="s">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>217</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" t="s">
         <v>241</v>
       </c>
       <c r="C19" s="1">
         <v>1236</v>
       </c>
-      <c r="D19" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="0" t="s">
+      <c r="D19" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>223</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" t="s">
         <v>241</v>
       </c>
       <c r="C20" s="1">
         <v>1399</v>
       </c>
-      <c r="D20" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="0" t="s">
+      <c r="D20" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>229</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" t="s">
         <v>241</v>
       </c>
       <c r="C21" s="1">
         <v>1802</v>
       </c>
-      <c r="D21" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="0" t="s">
+      <c r="D21" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>186</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="B22" t="s">
         <v>242</v>
       </c>
       <c r="C22" s="1">
         <v>259</v>
       </c>
-      <c r="D22" s="0" t="s">
+      <c r="D22" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="0" t="s">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>198</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" t="s">
         <v>242</v>
       </c>
       <c r="C23" s="1">
         <v>577</v>
       </c>
-      <c r="D23" s="0" t="s">
+      <c r="D23" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="0" t="s">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>210</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" t="s">
         <v>242</v>
       </c>
       <c r="C24" s="1">
         <v>1022</v>
       </c>
-      <c r="D24" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="0" t="s">
+      <c r="D24" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>182</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" t="s">
         <v>242</v>
       </c>
       <c r="C25" s="1">
         <v>142</v>
       </c>
-      <c r="D25" s="0" t="s">
+      <c r="D25" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="0" t="s">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>188</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="B26" t="s">
         <v>242</v>
       </c>
       <c r="C26" s="1">
         <v>301</v>
       </c>
-      <c r="D26" s="0" t="s">
+      <c r="D26" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="0" t="s">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>194</v>
       </c>
-      <c r="B27" s="0" t="s">
+      <c r="B27" t="s">
         <v>242</v>
       </c>
       <c r="C27" s="1">
         <v>453</v>
       </c>
-      <c r="D27" s="0" t="s">
+      <c r="D27" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="0" t="s">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>206</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="B28" t="s">
         <v>242</v>
       </c>
       <c r="C28" s="1">
         <v>951</v>
       </c>
-      <c r="D28" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="0" t="s">
+      <c r="D28" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>212</v>
       </c>
-      <c r="B29" s="0" t="s">
+      <c r="B29" t="s">
         <v>242</v>
       </c>
       <c r="C29" s="1">
         <v>1191</v>
       </c>
-      <c r="D29" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="0" t="s">
+      <c r="D29" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>218</v>
       </c>
-      <c r="B30" s="0" t="s">
+      <c r="B30" t="s">
         <v>242</v>
       </c>
       <c r="C30" s="1">
         <v>1236</v>
       </c>
-      <c r="D30" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="0" t="s">
+      <c r="D30" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>224</v>
       </c>
-      <c r="B31" s="0" t="s">
+      <c r="B31" t="s">
         <v>242</v>
       </c>
       <c r="C31" s="1">
         <v>1425</v>
       </c>
-      <c r="D31" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="0" t="s">
+      <c r="D31" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>230</v>
       </c>
-      <c r="B32" s="0" t="s">
+      <c r="B32" t="s">
         <v>242</v>
       </c>
       <c r="C32" s="1">
         <v>1816</v>
       </c>
-      <c r="D32" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="0" t="s">
+      <c r="D32" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>203</v>
       </c>
-      <c r="B33" s="0" t="s">
+      <c r="B33" t="s">
         <v>243</v>
       </c>
       <c r="C33" s="1">
         <v>722</v>
       </c>
-      <c r="D33" s="0" t="s">
+      <c r="D33" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="0" t="s">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>209</v>
       </c>
-      <c r="B34" s="0" t="s">
+      <c r="B34" t="s">
         <v>243</v>
       </c>
       <c r="C34" s="1">
         <v>1018</v>
       </c>
-      <c r="D34" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="0" t="s">
+      <c r="D34" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>216</v>
       </c>
-      <c r="B35" s="0" t="s">
+      <c r="B35" t="s">
         <v>243</v>
       </c>
       <c r="C35" s="1">
         <v>1218</v>
       </c>
-      <c r="D35" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="0" t="s">
+      <c r="D35" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>183</v>
       </c>
-      <c r="B36" s="0" t="s">
+      <c r="B36" t="s">
         <v>243</v>
       </c>
       <c r="C36" s="1">
         <v>166</v>
       </c>
-      <c r="D36" s="0" t="s">
+      <c r="D36" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="0" t="s">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>189</v>
       </c>
-      <c r="B37" s="0" t="s">
+      <c r="B37" t="s">
         <v>243</v>
       </c>
       <c r="C37" s="1">
         <v>322</v>
       </c>
-      <c r="D37" s="0" t="s">
+      <c r="D37" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="0" t="s">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>195</v>
       </c>
-      <c r="B38" s="0" t="s">
+      <c r="B38" t="s">
         <v>243</v>
       </c>
       <c r="C38" s="1">
         <v>467</v>
       </c>
-      <c r="D38" s="0" t="s">
+      <c r="D38" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="0" t="s">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>201</v>
       </c>
-      <c r="B39" s="0" t="s">
+      <c r="B39" t="s">
         <v>243</v>
       </c>
       <c r="C39" s="1">
         <v>656</v>
       </c>
-      <c r="D39" s="0" t="s">
+      <c r="D39" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="0" t="s">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>207</v>
       </c>
-      <c r="B40" s="0" t="s">
+      <c r="B40" t="s">
         <v>243</v>
       </c>
       <c r="C40" s="1">
         <v>1000</v>
       </c>
-      <c r="D40" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="0" t="s">
+      <c r="D40" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>213</v>
       </c>
-      <c r="B41" s="0" t="s">
+      <c r="B41" t="s">
         <v>243</v>
       </c>
       <c r="C41" s="1">
         <v>1208</v>
       </c>
-      <c r="D41" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="0" t="s">
+      <c r="D41" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>219</v>
       </c>
-      <c r="B42" s="0" t="s">
+      <c r="B42" t="s">
         <v>243</v>
       </c>
       <c r="C42" s="1">
         <v>1247</v>
       </c>
-      <c r="D42" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="0" t="s">
+      <c r="D42" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>225</v>
       </c>
-      <c r="B43" s="0" t="s">
+      <c r="B43" t="s">
         <v>243</v>
       </c>
       <c r="C43" s="1">
         <v>1456</v>
       </c>
-      <c r="D43" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="0" t="s">
+      <c r="D43" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>231</v>
       </c>
-      <c r="B44" s="0" t="s">
+      <c r="B44" t="s">
         <v>243</v>
       </c>
       <c r="C44" s="1">
         <v>1829</v>
       </c>
-      <c r="D44" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="0" t="s">
+      <c r="D44" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>232</v>
       </c>
-      <c r="B45" s="0" t="s">
+      <c r="B45" t="s">
         <v>243</v>
       </c>
       <c r="C45" s="1">
         <v>1841</v>
       </c>
-      <c r="D45" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="0" t="s">
+      <c r="D45" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>215</v>
       </c>
-      <c r="B46" s="0" t="s">
+      <c r="B46" t="s">
         <v>239</v>
       </c>
       <c r="C46" s="1">
         <v>1218</v>
       </c>
-      <c r="D46" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="0" t="s">
+      <c r="D46" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>180</v>
       </c>
-      <c r="B47" s="0" t="s">
+      <c r="B47" t="s">
         <v>239</v>
       </c>
       <c r="C47" s="1">
         <v>125</v>
       </c>
-      <c r="D47" s="0" t="s">
+      <c r="D47" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="0" t="s">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>172</v>
       </c>
-      <c r="B48" s="0" t="s">
+      <c r="B48" t="s">
         <v>239</v>
       </c>
       <c r="C48" s="1">
         <v>84</v>
       </c>
-      <c r="D48" s="0" t="s">
+      <c r="D48" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="0" t="s">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
         <v>184</v>
       </c>
-      <c r="B49" s="0" t="s">
+      <c r="B49" t="s">
         <v>239</v>
       </c>
       <c r="C49" s="1">
         <v>226</v>
       </c>
-      <c r="D49" s="0" t="s">
+      <c r="D49" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="0" t="s">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
         <v>190</v>
       </c>
-      <c r="B50" s="0" t="s">
+      <c r="B50" t="s">
         <v>239</v>
       </c>
       <c r="C50" s="1">
         <v>330</v>
       </c>
-      <c r="D50" s="0" t="s">
+      <c r="D50" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="0" t="s">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
         <v>196</v>
       </c>
-      <c r="B51" s="0" t="s">
+      <c r="B51" t="s">
         <v>239</v>
       </c>
       <c r="C51" s="1">
         <v>557</v>
       </c>
-      <c r="D51" s="0" t="s">
+      <c r="D51" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="0" t="s">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
         <v>202</v>
       </c>
-      <c r="B52" s="0" t="s">
+      <c r="B52" t="s">
         <v>239</v>
       </c>
       <c r="C52" s="1">
         <v>706</v>
       </c>
-      <c r="D52" s="0" t="s">
+      <c r="D52" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="0" t="s">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
         <v>208</v>
       </c>
-      <c r="B53" s="0" t="s">
+      <c r="B53" t="s">
         <v>239</v>
       </c>
       <c r="C53" s="1">
         <v>1001</v>
       </c>
-      <c r="D53" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="0" t="s">
+      <c r="D53" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
         <v>214</v>
       </c>
-      <c r="B54" s="0" t="s">
+      <c r="B54" t="s">
         <v>239</v>
       </c>
       <c r="C54" s="1">
         <v>1215</v>
       </c>
-      <c r="D54" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="0" t="s">
+      <c r="D54" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
         <v>220</v>
       </c>
-      <c r="B55" s="0" t="s">
+      <c r="B55" t="s">
         <v>239</v>
       </c>
       <c r="C55" s="1">
         <v>1256</v>
       </c>
-      <c r="D55" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="0" t="s">
+      <c r="D55" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
         <v>226</v>
       </c>
-      <c r="B56" s="0" t="s">
+      <c r="B56" t="s">
         <v>239</v>
       </c>
       <c r="C56" s="1">
         <v>1527</v>
       </c>
-      <c r="D56" s="0" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="0" t="s">
+      <c r="D56" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
         <v>233</v>
       </c>
-      <c r="B57" s="0" t="s">
+      <c r="B57" t="s">
         <v>239</v>
       </c>
       <c r="C57" s="1">
         <v>1906</v>
       </c>
-      <c r="D57" s="0" t="s">
+      <c r="D57" t="s">
         <v>177</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
   <tableParts count="2">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" ht="20.25">
-      <c r="A1" s="3" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="2" ht="15.75">
-      <c r="A2" s="0" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="0" t="s">
-        <v>246</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=EPPlusLicense.txt>This workbook was created with the EPPlus library, licensed to Alo1234 under the Polyform Noncommercial license, see https://polyformproject.org/licenses/noncommercial/1.0.0
-For more information about EPPlus, see https://epplussoftware.com/
-
 </file>
</xml_diff>